<commit_message>
June 4 2024 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0012451_VerifyCFIndustryGroupUpdatedToTECHonCompanies.xlsx
+++ b/TestData/LV_TMTT0012451_VerifyCFIndustryGroupUpdatedToTECHonCompanies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07AD1082-A35E-4313-A2A7-7BAF7CF3671F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC5AC693-3C89-4A5A-AF2A-41AA585A6B77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="0" showVerticalScroll="0" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView showHorizontalScroll="0" showVerticalScroll="0" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
@@ -20,10 +20,21 @@
     <sheet name="IndustryType" sheetId="1" r:id="rId5"/>
     <sheet name="Tabs" sheetId="10" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -478,11 +489,12 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyFont="0" applyBorder="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyFont="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -910,21 +922,66 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N12" s="4"/>
+      <c r="O12" s="4"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N13" s="4"/>
+      <c r="O13" s="4"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N14" s="4"/>
+      <c r="O14" s="4"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N15" s="4"/>
+      <c r="O15" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>

</xml_diff>